<commit_message>
API testing and debugging
</commit_message>
<xml_diff>
--- a/data/raw/maintenance/maintenance_log.xlsx
+++ b/data/raw/maintenance/maintenance_log.xlsx
@@ -455,7 +455,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LOG-82CD</t>
+          <t>LOG-661A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOG-375D</t>
+          <t>LOG-D51E</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -515,7 +515,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOG-AAA2</t>
+          <t>LOG-9E99</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LOG-4773</t>
+          <t>LOG-FC85</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LOG-81C3</t>
+          <t>LOG-295F</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -605,7 +605,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LOG-CA0D</t>
+          <t>LOG-6A4D</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LOG-0968</t>
+          <t>LOG-8023</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LOG-3BD9</t>
+          <t>LOG-25A5</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -695,7 +695,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LOG-D810</t>
+          <t>LOG-81CB</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -725,7 +725,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LOG-FFF2</t>
+          <t>LOG-F31B</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LOG-4FF5</t>
+          <t>LOG-7304</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -785,7 +785,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LOG-45D6</t>
+          <t>LOG-34CB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LOG-4349</t>
+          <t>LOG-DC56</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -845,7 +845,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LOG-DFF6</t>
+          <t>LOG-72E1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LOG-B49D</t>
+          <t>LOG-C67B</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -905,7 +905,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LOG-7E27</t>
+          <t>LOG-C87D</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LOG-0F19</t>
+          <t>LOG-B89B</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -965,7 +965,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LOG-978E</t>
+          <t>LOG-7620</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LOG-0B77</t>
+          <t>LOG-F236</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1025,7 +1025,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LOG-70D0</t>
+          <t>LOG-D404</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1055,7 +1055,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LOG-67D5</t>
+          <t>LOG-BD00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1085,7 +1085,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LOG-2876</t>
+          <t>LOG-9C73</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1115,7 +1115,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LOG-CAC7</t>
+          <t>LOG-AAB5</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1145,7 +1145,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LOG-DB21</t>
+          <t>LOG-32A4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1175,7 +1175,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LOG-CA7F</t>
+          <t>LOG-7650</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1205,7 +1205,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LOG-0732</t>
+          <t>LOG-E0EC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1235,7 +1235,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LOG-A620</t>
+          <t>LOG-2DB0</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1265,7 +1265,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LOG-E095</t>
+          <t>LOG-A873</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1295,7 +1295,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LOG-9352</t>
+          <t>LOG-454D</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1325,7 +1325,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LOG-7870</t>
+          <t>LOG-ECCB</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1355,7 +1355,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LOG-2FCC</t>
+          <t>LOG-3CC2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1385,7 +1385,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LOG-8AB2</t>
+          <t>LOG-1929</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1415,7 +1415,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LOG-3597</t>
+          <t>LOG-91EF</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1445,7 +1445,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LOG-2010</t>
+          <t>LOG-B10A</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1475,7 +1475,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LOG-4744</t>
+          <t>LOG-F67E</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1505,7 +1505,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LOG-0372</t>
+          <t>LOG-72B1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LOG-275A</t>
+          <t>LOG-C299</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1565,7 +1565,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LOG-E66B</t>
+          <t>LOG-3A4A</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1595,7 +1595,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LOG-5C04</t>
+          <t>LOG-8919</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1625,7 +1625,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LOG-4298</t>
+          <t>LOG-4D5C</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1655,7 +1655,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LOG-FACC</t>
+          <t>LOG-B793</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1685,7 +1685,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LOG-1369</t>
+          <t>LOG-1A77</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1715,7 +1715,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LOG-27DB</t>
+          <t>LOG-CE96</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1745,7 +1745,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LOG-11B3</t>
+          <t>LOG-A13E</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1775,7 +1775,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LOG-828C</t>
+          <t>LOG-F51E</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1805,7 +1805,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LOG-874A</t>
+          <t>LOG-5ED6</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1835,7 +1835,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LOG-62A1</t>
+          <t>LOG-C568</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1865,7 +1865,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LOG-EB71</t>
+          <t>LOG-EB7E</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1895,7 +1895,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LOG-BA1E</t>
+          <t>LOG-6D09</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1925,7 +1925,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LOG-2F1E</t>
+          <t>LOG-7605</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1955,7 +1955,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LOG-A24E</t>
+          <t>LOG-1862</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1985,7 +1985,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LOG-0778</t>
+          <t>LOG-FFC3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2015,7 +2015,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LOG-8903</t>
+          <t>LOG-821B</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2045,7 +2045,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LOG-6E89</t>
+          <t>LOG-4658</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2075,7 +2075,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LOG-2E2A</t>
+          <t>LOG-EA88</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2105,7 +2105,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LOG-B8FF</t>
+          <t>LOG-AB4D</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2135,7 +2135,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LOG-D59F</t>
+          <t>LOG-F38F</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2165,7 +2165,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LOG-3B49</t>
+          <t>LOG-BD91</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2195,7 +2195,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LOG-16EE</t>
+          <t>LOG-5311</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2225,7 +2225,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LOG-4C79</t>
+          <t>LOG-FCDC</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">

</xml_diff>

<commit_message>
Add RAG knowledge base document upload feature
</commit_message>
<xml_diff>
--- a/data/raw/maintenance/maintenance_log.xlsx
+++ b/data/raw/maintenance/maintenance_log.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,32 +433,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Log_ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Pump_ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Event_Timestamp</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Event_Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Failed_Component</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Root_Cause</t>
         </is>
@@ -455,7 +467,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LOG-661A</t>
+          <t>LOG-CCE5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,7 +475,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,7 +497,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOG-D51E</t>
+          <t>LOG-5B44</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +505,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -515,7 +527,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOG-9E99</t>
+          <t>LOG-EDB3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -523,7 +535,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -545,7 +557,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LOG-FC85</t>
+          <t>LOG-F250</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -553,7 +565,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -575,7 +587,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LOG-295F</t>
+          <t>LOG-C9AF</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -583,7 +595,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C6" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -605,7 +617,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LOG-6A4D</t>
+          <t>LOG-A0CB</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -613,7 +625,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C7" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -635,7 +647,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LOG-8023</t>
+          <t>LOG-1116</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -643,7 +655,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -665,7 +677,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LOG-25A5</t>
+          <t>LOG-01E5</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -673,7 +685,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C9" s="1" t="n">
+      <c r="C9" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -695,7 +707,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LOG-81CB</t>
+          <t>LOG-BF72</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -703,7 +715,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -725,7 +737,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LOG-F31B</t>
+          <t>LOG-6377</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -733,7 +745,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="2" t="n">
         <v>46202</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -755,7 +767,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LOG-7304</t>
+          <t>LOG-B0E9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -763,7 +775,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C12" s="1" t="n">
+      <c r="C12" s="2" t="n">
         <v>46292</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -785,7 +797,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LOG-34CB</t>
+          <t>LOG-61B0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -793,7 +805,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C13" s="1" t="n">
+      <c r="C13" s="2" t="n">
         <v>46292</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -815,7 +827,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LOG-DC56</t>
+          <t>LOG-EAC9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -823,7 +835,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C14" s="1" t="n">
+      <c r="C14" s="2" t="n">
         <v>46292</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -845,7 +857,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LOG-72E1</t>
+          <t>LOG-8F2C</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -853,7 +865,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C15" s="1" t="n">
+      <c r="C15" s="2" t="n">
         <v>46292</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -875,7 +887,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LOG-C67B</t>
+          <t>LOG-29A8</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -883,7 +895,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C16" s="1" t="n">
+      <c r="C16" s="2" t="n">
         <v>46292</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -905,7 +917,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LOG-C87D</t>
+          <t>LOG-9D6C</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -913,7 +925,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C17" s="1" t="n">
+      <c r="C17" s="2" t="n">
         <v>46382</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -935,7 +947,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LOG-B89B</t>
+          <t>LOG-73A8</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -943,7 +955,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C18" s="1" t="n">
+      <c r="C18" s="2" t="n">
         <v>46382</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -965,7 +977,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LOG-7620</t>
+          <t>LOG-16A7</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -973,7 +985,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C19" s="2" t="n">
         <v>46382</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -995,7 +1007,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LOG-F236</t>
+          <t>LOG-A503</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1003,7 +1015,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="2" t="n">
         <v>46382</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -1025,7 +1037,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LOG-D404</t>
+          <t>LOG-6F86</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1033,7 +1045,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C21" s="1" t="n">
+      <c r="C21" s="2" t="n">
         <v>46382</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -1055,7 +1067,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LOG-BD00</t>
+          <t>LOG-1A62</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1063,7 +1075,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C22" s="1" t="n">
+      <c r="C22" s="2" t="n">
         <v>46472</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -1085,7 +1097,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LOG-9C73</t>
+          <t>LOG-33D2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1093,7 +1105,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C23" s="1" t="n">
+      <c r="C23" s="2" t="n">
         <v>46472</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -1115,7 +1127,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LOG-AAB5</t>
+          <t>LOG-459B</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1123,7 +1135,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C24" s="1" t="n">
+      <c r="C24" s="2" t="n">
         <v>46472</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -1145,7 +1157,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LOG-32A4</t>
+          <t>LOG-EB4C</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1153,7 +1165,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C25" s="1" t="n">
+      <c r="C25" s="2" t="n">
         <v>46472</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -1175,7 +1187,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LOG-7650</t>
+          <t>LOG-E64C</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1183,7 +1195,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C26" s="1" t="n">
+      <c r="C26" s="2" t="n">
         <v>46472</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -1205,7 +1217,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LOG-E0EC</t>
+          <t>LOG-2C17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1213,7 +1225,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C27" s="1" t="n">
+      <c r="C27" s="2" t="n">
         <v>46562</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -1235,7 +1247,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LOG-2DB0</t>
+          <t>LOG-67D1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1243,7 +1255,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C28" s="1" t="n">
+      <c r="C28" s="2" t="n">
         <v>46562</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -1265,7 +1277,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LOG-A873</t>
+          <t>LOG-7BFB</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1273,7 +1285,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C29" s="1" t="n">
+      <c r="C29" s="2" t="n">
         <v>46562</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -1295,7 +1307,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LOG-454D</t>
+          <t>LOG-0483</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1303,7 +1315,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C30" s="1" t="n">
+      <c r="C30" s="2" t="n">
         <v>46562</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -1325,7 +1337,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LOG-ECCB</t>
+          <t>LOG-0715</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1333,7 +1345,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C31" s="1" t="n">
+      <c r="C31" s="2" t="n">
         <v>46562</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -1355,7 +1367,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LOG-3CC2</t>
+          <t>LOG-7428</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1363,7 +1375,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C32" s="1" t="n">
+      <c r="C32" s="2" t="n">
         <v>46652</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -1385,7 +1397,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LOG-1929</t>
+          <t>LOG-2B1B</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1393,7 +1405,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C33" s="1" t="n">
+      <c r="C33" s="2" t="n">
         <v>46652</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -1415,7 +1427,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LOG-91EF</t>
+          <t>LOG-79DF</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1423,7 +1435,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C34" s="1" t="n">
+      <c r="C34" s="2" t="n">
         <v>46652</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -1445,7 +1457,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LOG-B10A</t>
+          <t>LOG-801F</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1453,7 +1465,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C35" s="1" t="n">
+      <c r="C35" s="2" t="n">
         <v>46652</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -1475,7 +1487,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LOG-F67E</t>
+          <t>LOG-91C0</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1483,7 +1495,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C36" s="1" t="n">
+      <c r="C36" s="2" t="n">
         <v>46652</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -1505,7 +1517,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LOG-72B1</t>
+          <t>LOG-26E4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1513,7 +1525,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C37" s="1" t="n">
+      <c r="C37" s="2" t="n">
         <v>46742</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -1535,7 +1547,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LOG-C299</t>
+          <t>LOG-7832</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1543,7 +1555,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C38" s="1" t="n">
+      <c r="C38" s="2" t="n">
         <v>46742</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -1565,7 +1577,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LOG-3A4A</t>
+          <t>LOG-1B92</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1573,7 +1585,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C39" s="1" t="n">
+      <c r="C39" s="2" t="n">
         <v>46742</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -1595,7 +1607,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LOG-8919</t>
+          <t>LOG-46B0</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1603,7 +1615,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C40" s="1" t="n">
+      <c r="C40" s="2" t="n">
         <v>46742</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -1625,7 +1637,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LOG-4D5C</t>
+          <t>LOG-23CA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1633,7 +1645,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C41" s="1" t="n">
+      <c r="C41" s="2" t="n">
         <v>46742</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -1655,7 +1667,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LOG-B793</t>
+          <t>LOG-20D1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1663,7 +1675,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C42" s="1" t="n">
+      <c r="C42" s="2" t="n">
         <v>46832</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -1685,7 +1697,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LOG-1A77</t>
+          <t>LOG-68CA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1693,7 +1705,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C43" s="1" t="n">
+      <c r="C43" s="2" t="n">
         <v>46832</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -1715,7 +1727,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LOG-CE96</t>
+          <t>LOG-9FDD</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1723,7 +1735,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C44" s="1" t="n">
+      <c r="C44" s="2" t="n">
         <v>46832</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -1745,7 +1757,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LOG-A13E</t>
+          <t>LOG-3ACE</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1753,7 +1765,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C45" s="1" t="n">
+      <c r="C45" s="2" t="n">
         <v>46832</v>
       </c>
       <c r="D45" t="inlineStr">
@@ -1775,7 +1787,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LOG-F51E</t>
+          <t>LOG-372B</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1783,7 +1795,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C46" s="1" t="n">
+      <c r="C46" s="2" t="n">
         <v>46832</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -1805,7 +1817,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LOG-5ED6</t>
+          <t>LOG-29F9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1813,7 +1825,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C47" s="1" t="n">
+      <c r="C47" s="2" t="n">
         <v>46922</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -1835,7 +1847,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LOG-C568</t>
+          <t>LOG-D3C8</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1843,7 +1855,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C48" s="1" t="n">
+      <c r="C48" s="2" t="n">
         <v>46922</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -1865,7 +1877,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LOG-EB7E</t>
+          <t>LOG-F887</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1873,7 +1885,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C49" s="1" t="n">
+      <c r="C49" s="2" t="n">
         <v>46922</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -1895,7 +1907,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LOG-6D09</t>
+          <t>LOG-B043</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1903,7 +1915,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C50" s="1" t="n">
+      <c r="C50" s="2" t="n">
         <v>46922</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -1925,7 +1937,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LOG-7605</t>
+          <t>LOG-4418</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1933,7 +1945,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C51" s="1" t="n">
+      <c r="C51" s="2" t="n">
         <v>46922</v>
       </c>
       <c r="D51" t="inlineStr">
@@ -1955,7 +1967,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LOG-1862</t>
+          <t>LOG-3118</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1963,7 +1975,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C52" s="1" t="n">
+      <c r="C52" s="2" t="n">
         <v>47012</v>
       </c>
       <c r="D52" t="inlineStr">
@@ -1985,7 +1997,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LOG-FFC3</t>
+          <t>LOG-6650</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1993,7 +2005,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C53" s="1" t="n">
+      <c r="C53" s="2" t="n">
         <v>47012</v>
       </c>
       <c r="D53" t="inlineStr">
@@ -2015,7 +2027,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LOG-821B</t>
+          <t>LOG-6C4F</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2023,7 +2035,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C54" s="1" t="n">
+      <c r="C54" s="2" t="n">
         <v>47012</v>
       </c>
       <c r="D54" t="inlineStr">
@@ -2045,7 +2057,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LOG-4658</t>
+          <t>LOG-3690</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2053,7 +2065,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C55" s="1" t="n">
+      <c r="C55" s="2" t="n">
         <v>47012</v>
       </c>
       <c r="D55" t="inlineStr">
@@ -2075,7 +2087,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LOG-EA88</t>
+          <t>LOG-F6AE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2083,7 +2095,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C56" s="1" t="n">
+      <c r="C56" s="2" t="n">
         <v>47012</v>
       </c>
       <c r="D56" t="inlineStr">
@@ -2105,7 +2117,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LOG-AB4D</t>
+          <t>LOG-0400</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2113,7 +2125,7 @@
           <t>KSB-CALIO-3040-1003</t>
         </is>
       </c>
-      <c r="C57" s="1" t="n">
+      <c r="C57" s="2" t="n">
         <v>47102</v>
       </c>
       <c r="D57" t="inlineStr">
@@ -2135,7 +2147,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LOG-F38F</t>
+          <t>LOG-ECA3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2143,7 +2155,7 @@
           <t>KSB-CALIO-3040-1001</t>
         </is>
       </c>
-      <c r="C58" s="1" t="n">
+      <c r="C58" s="2" t="n">
         <v>47102</v>
       </c>
       <c r="D58" t="inlineStr">
@@ -2165,7 +2177,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LOG-BD91</t>
+          <t>LOG-D245</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2173,7 +2185,7 @@
           <t>KSB-CALIO-3040-1000</t>
         </is>
       </c>
-      <c r="C59" s="1" t="n">
+      <c r="C59" s="2" t="n">
         <v>47102</v>
       </c>
       <c r="D59" t="inlineStr">
@@ -2195,7 +2207,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LOG-5311</t>
+          <t>LOG-842F</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2203,7 +2215,7 @@
           <t>KSB-CALIO-3040-1002</t>
         </is>
       </c>
-      <c r="C60" s="1" t="n">
+      <c r="C60" s="2" t="n">
         <v>47102</v>
       </c>
       <c r="D60" t="inlineStr">
@@ -2225,7 +2237,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LOG-FCDC</t>
+          <t>LOG-4AF0</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2233,7 +2245,7 @@
           <t>KSB-CALIO-3040-1004</t>
         </is>
       </c>
-      <c r="C61" s="1" t="n">
+      <c r="C61" s="2" t="n">
         <v>47102</v>
       </c>
       <c r="D61" t="inlineStr">

</xml_diff>